<commit_message>
Add GitHub Pages workflow
</commit_message>
<xml_diff>
--- a/Input text AAA.xlsx
+++ b/Input text AAA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heal_\Documents\GitHub\henrikalmquist.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B1F4DB-1A9D-4336-AA92-1521FB9E9132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4AE5A1-4BD8-4A84-98F0-975C3BD2AC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="18220" activeTab="4" xr2:uid="{75645F56-5FAC-422B-9288-0CDC3C429DEC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="105">
   <si>
     <t>Index</t>
   </si>
@@ -342,20 +342,6 @@
     <t>AAA000/AAA00.jpg</t>
   </si>
   <si>
-    <t>Clients: [Riksbyggen](https://www.riksbyggen.se), [Lund City](https://en.lundcity.se/), [Växjö Municipality](https://www.vaxjo.se/), [The Ministry for Europe and Foreign Affairs France](https://www.diplomatie.gouv.fr/en/), [Malmö Stad](malmö.se) and private. 
-Collaborations: [MOD Group](https://www.modgroup.se/), [Draken Arkitektur](https://drakenarkitektur.se/), [Outer Space Landscape Architecture](https://outerspacearkitekter.se/), [Blick Arkitektur](https://www.blickarkitektur.se/), [Wingård Arkitektkontor](https://www.wingardhs.se), [LTH](https://www.arch.lth.se/), [KTH](https://www.kth.se/en/abe), [Rambøll Group](https://www.ramboll.com/), [Djernes &amp; Bell](https://djernesbell.com/en), [Grip+Torarp](https://www.griptorarp.com/), [Malmö universitet](https://mau.se/forskning/forskningsamnen/urbana-studier/), [Contexo Studio](https://www.contexo.studio/), [Studio 1836](https://www.studio1836.fr/).
-Presentations: [Form Design Center Skåne](https://formdesigncenter.com/), [TU Graz](https://www.tugraz.at/en/fakultaeten/architektur/home), [Krook &amp; Tjäder Arkitekter](http://www.krook.tjader.se/), [Sällskapet för restaurering](https://sallskapet.eu/). 
-Publications: [Arkitektur](https://arkitektur.se/), [Rum](https://www.byrum.se/kategori/arkitektur/), [Arkitekten](https://arkitekten.se/), [Kritik](https://syntesforlag.blogspot.com/), [Plan](https://www.planering.org/om-plan), [Utkast](http://faltstudio.com/).
-AAA is a Swedish shareholder company with the organisation number 556574-6152, formerly Almquist Architecture Agency AB. © 2025 Agency for Adaptive Architecture. All rights reserved.</t>
-  </si>
-  <si>
-    <t>Kunder: [Riksbyggen](https://www.riksbyggen.se), [Lund City](https://en.lundcity.se/), [Växjö Municipality](https://www.vaxjo.se/), [The Ministry for Europe and Foreign Affairs France](https://www.diplomatie.gouv.fr/en/), [Malmö Stad](malmö.se) och privat. 
-Samarbeten: [MOD Group](https://www.modgroup.se/), [Draken Arkitektur](https://drakenarkitektur.se/), [Outer Space Landscape Architecture](https://outerspacearkitekter.se/), [Blick Arkitektur](https://www.blickarkitektur.se/), [Wingård Arkitektkontor](https://www.wingardhs.se), [LTH](https://www.arch.lth.se/), [KTH](https://www.kth.se/en/abe), [Rambøll Group](https://www.ramboll.com/), [Djernes &amp; Bell](https://djernesbell.com/en), [Grip+Torarp](https://www.griptorarp.com/), [Malmö universitet](https://mau.se/forskning/forskningsamnen/urbana-studier/), [Contexo Studio](https://www.contexo.studio/), [Studio 1836](https://www.studio1836.fr/).
-Presentationer: [Form Design Center Skåne](https://formdesigncenter.com/), [TU Graz](https://www.tugraz.at/en/fakultaeten/architektur/home), [Krook &amp; Tjäder Arkitekter](http://www.krook.tjader.se/), [Sällskapet för restaurering](https://sallskapet.eu/). 
-Publikationer: [Arkitektur](https://arkitektur.se/), [Rum](https://www.byrum.se/kategori/arkitektur/), [Arkitekten](https://arkitekten.se/), [Kritik](https://syntesforlag.blogspot.com/), [Plan](https://www.planering.org/om-plan).
-AAA är ett svenskt aktiebolag med organisationsnummer 556574-6152, tidigare Almquist Architecture Agency AB. © 2025 Agency for Adaptive Architecture. Alla rättigheter reserverade.</t>
-  </si>
-  <si>
     <t>Practice, research and policy</t>
   </si>
   <si>
@@ -374,9 +360,6 @@
   </si>
   <si>
     <t>Henrik Almquist, Arkitekt SAR/MSA, Dip. d’État (France)</t>
-  </si>
-  <si>
-    <t>Funded AAA 2024, bringing experience from Stockholm, Paris and Tokyo. He has carried out projects from  in-situ dialogues to early design proposals to seeing through the construction. Henrik teaches at Lund University where he directs the masterstudio Act of Altering and he is an active voice in the ongoing dialogue on the existing environment and sustainability.</t>
   </si>
   <si>
     <t>**Varje byggnad, varje situation, rymmer en dold potential**. AAA:s roll som arkitekter är att identifiera och lyfta fram dessa kvaliteter. Oavsett om det rör sig om en enskild byggnad eller ett helt stadsområde, kan små justeringar skapa en betydande inverkan och förändra hur ett utrymme känns och fungerar. AAA:s tillvägagångssätt bygger på att lyssna och lära, för att skapa strategier och design som harmoniserar med omgivningen och svarar mot varje kunds unika behov.
@@ -413,6 +396,29 @@
 * AAA bjuds återkommande in för att tala om utvecklingen av praktiken och hållbara strategier för stadsplanering.
 Varje byggnad och plats presenterar sitt unika fall; metoder måste skräddarsys efter dess specifika behov och potential.
 **Att navigera i denna skärningspunkt mellan ekonomi och ekologi, kultur och teknik, är AAA:s expertis.**</t>
+  </si>
+  <si>
+    <t>Founded AAA 2024, bringing experience from Stockholm, Paris and Tokyo. He has carried out projects from  in-situ dialogues to early design proposals to seeing through the construction. Henrik teaches at Lund University where he directs the masterstudio Act of Altering and he is an active voice in the ongoing dialogue on the existing environment and sustainability.</t>
+  </si>
+  <si>
+    <t>Clients: [Riksbyggen](https://www.riksbyggen.se), [Lund City](https://en.lundcity.se/), [Växjö Municipality](https://www.vaxjo.se/), [The Ministry for Europe and Foreign Affairs France](https://www.diplomatie.gouv.fr/en/), [Malmö Stad](malmö.se) and private. 
+Collaborations: [MOD Group](https://www.modgroup.se/), [Draken Arkitektur](https://drakenarkitektur.se/), [Outer Space Landscape Architecture](https://outerspacearkitekter.se/), [Blick Arkitektur](https://www.blickarkitektur.se/), [Wingård Arkitektkontor](https://www.wingardhs.se), [LTH](https://www.arch.lth.se/), [KTH](https://www.kth.se/en/abe), [Rambøll Group](https://www.ramboll.com/), [Djernes &amp; Bell](https://djernesbell.com/en), [Grip+Torarp](https://www.griptorarp.com/), [Malmö universitet](https://mau.se/forskning/forskningsamnen/urbana-studier/), [Contexo Studio](https://www.contexo.studio/), [Studio 1836](https://www.studio1836.fr/).
+Presentations: [Form Design Center Skåne](https://formdesigncenter.com/), [TU Graz](https://www.tugraz.at/en/fakultaeten/architektur/home), [Krook &amp; Tjäder Arkitekter](http://www.krook.tjader.se/), [Sällskapet för restaurering](https://sallskapet.eu/). 
+Publications: [Arkitektur](https://arkitektur.se/), [Rum](https://www.byrum.se/kategori/arkitektur/), [Arkitekten](https://arkitekten.se/), [Kritik](https://syntesforlag.blogspot.com/), [Aftonbladet](https://www.aftonbladet.se/debatt/a/0VKpxB/acan-sverige-fullt-fungerande-hus-rivs-i-jakt-pa-vinst), [Plan](https://www.planering.org/om-plan), [Utkast](http://faltstudio.com/).
+AAA is a Swedish shareholder company with the organisation number 556574-6152, formerly Almquist Architecture Agency AB. © 2025 Agency for Adaptive Architecture. All rights reserved.</t>
+  </si>
+  <si>
+    <t>Kunder: [Riksbyggen](https://www.riksbyggen.se), [Lund City](https://en.lundcity.se/), [Växjö Municipality](https://www.vaxjo.se/), [The Ministry for Europe and Foreign Affairs France](https://www.diplomatie.gouv.fr/en/), [Malmö Stad](malmö.se) och privat. 
+Samarbeten: [MOD Group](https://www.modgroup.se/), [Draken Arkitektur](https://drakenarkitektur.se/), [Outer Space Landscape Architecture](https://outerspacearkitekter.se/), [Blick Arkitektur](https://www.blickarkitektur.se/), [Wingård Arkitektkontor](https://www.wingardhs.se), [LTH](https://www.arch.lth.se/), [KTH](https://www.kth.se/en/abe), [Rambøll Group](https://www.ramboll.com/), [Djernes &amp; Bell](https://djernesbell.com/en), [Grip+Torarp](https://www.griptorarp.com/), [Malmö universitet](https://mau.se/forskning/forskningsamnen/urbana-studier/), [Contexo Studio](https://www.contexo.studio/), [Studio 1836](https://www.studio1836.fr/).
+Presentationer: [Form Design Center Skåne](https://formdesigncenter.com/), [TU Graz](https://www.tugraz.at/en/fakultaeten/architektur/home), [Krook &amp; Tjäder Arkitekter](http://www.krook.tjader.se/), [Sällskapet för restaurering](https://sallskapet.eu/). 
+Publikationer: [Arkitektur](https://arkitektur.se/), [Rum](https://www.byrum.se/kategori/arkitektur/), [Arkitekten](https://arkitekten.se/), [Kritik](https://syntesforlag.blogspot.com/), [Aftonbladet](https://www.aftonbladet.se/debatt/a/0VKpxB/acan-sverige-fullt-fungerande-hus-rivs-i-jakt-pa-vinst), [Plan](https://www.planering.org/om-plan), [Utkast](http://faltstudio.com/).
+AAA är ett svenskt aktiebolag med organisationsnummer 556574-6152, tidigare Almquist Architecture Agency AB. © 2025 Agency for Adaptive Architecture. Alla rättigheter reserverade.</t>
+  </si>
+  <si>
+    <t>artiklar länkar</t>
+  </si>
+  <si>
+    <t>https://www.aftonbladet.se/debatt/a/0VKpxB/acan-sverige-fullt-fungerande-hus-rivs-i-jakt-pa-vinst</t>
   </si>
 </sst>
 </file>
@@ -8989,10 +8995,10 @@
         <v>51</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>86</v>
@@ -9012,10 +9018,10 @@
         <v>60</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>53</v>
@@ -11438,10 +11444,10 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>79</v>
@@ -11453,16 +11459,16 @@
         <v>82</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>83</v>
@@ -11478,10 +11484,10 @@
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -11491,16 +11497,16 @@
         <v>22</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2">
@@ -11564,8 +11570,12 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>

</xml_diff>